<commit_message>
Actualización automática ERP - Pedidos Pendientes - 06/10/2026 09:23:17
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCC69509-E9B3-48CD-BAF0-7344B0F422ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5CAA5B9E-F7F4-4ADC-8343-2D218965F77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{CB4ED01F-5C82-48F2-B805-4C82FE69C050}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{290B7EA0-DFA6-48E6-BD0B-34E71E281D80}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -5876,7 +5876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D612BB15-C4FF-477D-9DFA-4B3D796753FE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EDB18B4-1436-4FF3-918C-1070269E5BE9}">
   <dimension ref="A1:BI431"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 15/10/2026 06:28:01
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2BBECC2-BFE3-430C-8D9F-4E24870946CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{52A34435-B436-4E1D-9253-44920DD936E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{84D5DC18-C1A9-4AF6-AB8D-0C84C5E0C0E9}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{09A82D10-8AE2-44D7-9565-7EB8BA8D055C}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4432,7 +4432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{252BB1C4-7261-4E12-A4E7-43F5EECDA5C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DBD5CFF-7617-4E37-A568-903A3A165130}">
   <dimension ref="A1:BI296"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 15/10/2026 14:45:48
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A1FADDB-ABC8-4F2B-9E38-E92416ECB681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E054AF55-F871-4243-9C04-2CB33AE80589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21615" yWindow="1125" windowWidth="21600" windowHeight="11835" xr2:uid="{F9DDBBEC-B72D-4B01-AF56-C65B8AAD3EC4}"/>
+    <workbookView xWindow="21615" yWindow="1125" windowWidth="21600" windowHeight="11835" xr2:uid="{65D9C092-02CF-4740-AA31-D62055CDB2FA}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4281,7 +4281,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B5C8096-829E-497F-A5C0-673B5E979714}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F164A95-C55E-4F85-A026-A8E384589E3C}">
   <dimension ref="A1:BI274"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 15/10/2026 16:04:38
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E054AF55-F871-4243-9C04-2CB33AE80589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DE8C241-0F91-4648-8405-7640CB1C1DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21615" yWindow="1125" windowWidth="21600" windowHeight="11835" xr2:uid="{65D9C092-02CF-4740-AA31-D62055CDB2FA}"/>
+    <workbookView xWindow="21615" yWindow="1125" windowWidth="21600" windowHeight="11835" xr2:uid="{A6BCC0ED-D0B6-4F38-AC7A-36E7EBA63243}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4281,7 +4281,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F164A95-C55E-4F85-A026-A8E384589E3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96720F59-A336-4E4F-9460-686EB0D83E52}">
   <dimension ref="A1:BI274"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 16/10/2026 06:09:54
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{001DAB5D-154E-460D-A70D-0F75B0FC0F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{814DE409-164D-4769-9E2E-83C314A38A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3EF77943-7E84-4978-9B36-41C72D9AA55F}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{115FF9B9-0E00-4C58-A2DA-4F08C1D1C5EB}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4146,7 +4146,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A3F8DAD-0A8C-478B-B34D-28C37EFD645A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9502475D-03DA-4873-8148-D21F10048DEF}">
   <dimension ref="A1:BI269"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 20/10/2026 06:00:38
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{334667AE-1EA5-4D56-AD0B-02301202C71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{236FEA95-A301-4C02-B403-F1D66C0D0CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{649DAD8E-C413-40A7-95CB-995C344E32F0}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{19D9C6EB-132C-4615-A6E4-91942458F590}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4969,7 +4969,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34B3FC0D-8E90-417C-93E6-4DB4A10F0C59}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559B08A0-DF43-43FB-86E4-9A5B4C0964FC}">
   <dimension ref="A1:BI342"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 26/10/2026 06:05:29
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16C9645F-79C9-4CA0-91D5-022DA86009FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{66184A46-681E-42E8-8680-33606F0453DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{106DD25F-07AF-445B-8716-DD83B07BA890}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{2876516E-3B3C-45BC-A0C6-EFBA45632A9A}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4799,7 +4799,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2489E9C3-70C2-4104-90A8-43E8007D0580}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFEFC100-3DD0-426F-B69E-9437BF9CF621}">
   <dimension ref="A1:BI345"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -5005,10 +5005,10 @@
         <v>65</v>
       </c>
       <c r="F2">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G2">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H2" t="s">
         <v>66</v>
@@ -5190,7 +5190,7 @@
         <v>86</v>
       </c>
       <c r="F3">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G3">
         <v>7</v>
@@ -5375,10 +5375,10 @@
         <v>99</v>
       </c>
       <c r="F4">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G4">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H4" t="s">
         <v>100</v>
@@ -5560,10 +5560,10 @@
         <v>109</v>
       </c>
       <c r="F5">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G5">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H5" t="s">
         <v>87</v>
@@ -5745,10 +5745,10 @@
         <v>112</v>
       </c>
       <c r="F6">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H6" t="s">
         <v>113</v>
@@ -5930,7 +5930,7 @@
         <v>124</v>
       </c>
       <c r="F7">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G7">
         <v>27</v>
@@ -6115,10 +6115,10 @@
         <v>130</v>
       </c>
       <c r="F8">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G8">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H8" t="s">
         <v>131</v>
@@ -6300,10 +6300,10 @@
         <v>130</v>
       </c>
       <c r="F9">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G9">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H9" t="s">
         <v>139</v>
@@ -6485,10 +6485,10 @@
         <v>144</v>
       </c>
       <c r="F10">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G10">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H10" t="s">
         <v>87</v>
@@ -6670,10 +6670,10 @@
         <v>147</v>
       </c>
       <c r="F11">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G11">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H11" t="s">
         <v>148</v>
@@ -6855,10 +6855,10 @@
         <v>146</v>
       </c>
       <c r="F12">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G12">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H12" t="s">
         <v>113</v>
@@ -7040,10 +7040,10 @@
         <v>160</v>
       </c>
       <c r="F13">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G13">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H13" t="s">
         <v>161</v>
@@ -7225,10 +7225,10 @@
         <v>160</v>
       </c>
       <c r="F14">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G14">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H14" t="s">
         <v>161</v>
@@ -7410,10 +7410,10 @@
         <v>160</v>
       </c>
       <c r="F15">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G15">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H15" t="s">
         <v>170</v>
@@ -7595,10 +7595,10 @@
         <v>176</v>
       </c>
       <c r="F16">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G16">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H16" t="s">
         <v>177</v>
@@ -7780,10 +7780,10 @@
         <v>188</v>
       </c>
       <c r="F17">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G17">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H17" t="s">
         <v>189</v>
@@ -7965,10 +7965,10 @@
         <v>198</v>
       </c>
       <c r="F18">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G18">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H18" t="s">
         <v>199</v>
@@ -8150,10 +8150,10 @@
         <v>202</v>
       </c>
       <c r="F19">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G19">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H19" t="s">
         <v>203</v>
@@ -8335,10 +8335,10 @@
         <v>202</v>
       </c>
       <c r="F20">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G20">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H20" t="s">
         <v>211</v>
@@ -8520,7 +8520,7 @@
         <v>219</v>
       </c>
       <c r="F21">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G21">
         <v>13</v>
@@ -8705,7 +8705,7 @@
         <v>219</v>
       </c>
       <c r="F22">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -8890,10 +8890,10 @@
         <v>219</v>
       </c>
       <c r="F23">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G23">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H23" t="s">
         <v>222</v>
@@ -9075,10 +9075,10 @@
         <v>229</v>
       </c>
       <c r="F24">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G24">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H24" t="s">
         <v>230</v>
@@ -9260,10 +9260,10 @@
         <v>229</v>
       </c>
       <c r="F25">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G25">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H25" t="s">
         <v>236</v>
@@ -9445,10 +9445,10 @@
         <v>245</v>
       </c>
       <c r="F26">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G26">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H26" t="s">
         <v>246</v>
@@ -9630,10 +9630,10 @@
         <v>244</v>
       </c>
       <c r="F27">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G27">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H27" t="s">
         <v>254</v>
@@ -9815,10 +9815,10 @@
         <v>245</v>
       </c>
       <c r="F28">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G28">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H28" t="s">
         <v>263</v>
@@ -10000,10 +10000,10 @@
         <v>269</v>
       </c>
       <c r="F29">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G29">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H29" t="s">
         <v>270</v>
@@ -10185,10 +10185,10 @@
         <v>269</v>
       </c>
       <c r="F30">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G30">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H30" t="s">
         <v>170</v>
@@ -10370,10 +10370,10 @@
         <v>269</v>
       </c>
       <c r="F31">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G31">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H31" t="s">
         <v>87</v>
@@ -10555,10 +10555,10 @@
         <v>279</v>
       </c>
       <c r="F32">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G32">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H32" t="s">
         <v>280</v>
@@ -10740,10 +10740,10 @@
         <v>279</v>
       </c>
       <c r="F33">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G33">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H33" t="s">
         <v>287</v>
@@ -10925,10 +10925,10 @@
         <v>279</v>
       </c>
       <c r="F34">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G34">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H34" t="s">
         <v>291</v>
@@ -11110,7 +11110,7 @@
         <v>300</v>
       </c>
       <c r="F35">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G35">
         <v>7</v>
@@ -11295,10 +11295,10 @@
         <v>300</v>
       </c>
       <c r="F36">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G36">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H36" t="s">
         <v>311</v>
@@ -11480,10 +11480,10 @@
         <v>320</v>
       </c>
       <c r="F37">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G37">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H37" t="s">
         <v>321</v>
@@ -11665,10 +11665,10 @@
         <v>320</v>
       </c>
       <c r="F38">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G38">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H38" t="s">
         <v>327</v>
@@ -11850,10 +11850,10 @@
         <v>320</v>
       </c>
       <c r="F39">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G39">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H39" t="s">
         <v>330</v>
@@ -12035,10 +12035,10 @@
         <v>335</v>
       </c>
       <c r="F40">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G40">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H40" t="s">
         <v>287</v>
@@ -12220,10 +12220,10 @@
         <v>335</v>
       </c>
       <c r="F41">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G41">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H41" t="s">
         <v>337</v>
@@ -12405,10 +12405,10 @@
         <v>335</v>
       </c>
       <c r="F42">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G42">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H42" t="s">
         <v>342</v>
@@ -12590,10 +12590,10 @@
         <v>335</v>
       </c>
       <c r="F43">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G43">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H43" t="s">
         <v>345</v>
@@ -12775,10 +12775,10 @@
         <v>335</v>
       </c>
       <c r="F44">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G44">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H44" t="s">
         <v>352</v>
@@ -12960,10 +12960,10 @@
         <v>358</v>
       </c>
       <c r="F45">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G45">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H45" t="s">
         <v>359</v>
@@ -13145,10 +13145,10 @@
         <v>358</v>
       </c>
       <c r="F46">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G46">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H46" t="s">
         <v>363</v>
@@ -13330,10 +13330,10 @@
         <v>358</v>
       </c>
       <c r="F47">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G47">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H47" t="s">
         <v>369</v>
@@ -13515,10 +13515,10 @@
         <v>358</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G48">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H48" t="s">
         <v>374</v>
@@ -13700,10 +13700,10 @@
         <v>380</v>
       </c>
       <c r="F49">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G49">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H49" t="s">
         <v>113</v>
@@ -13885,10 +13885,10 @@
         <v>358</v>
       </c>
       <c r="F50">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G50">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H50" t="s">
         <v>382</v>
@@ -14070,10 +14070,10 @@
         <v>358</v>
       </c>
       <c r="F51">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G51">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H51" t="s">
         <v>391</v>
@@ -14255,10 +14255,10 @@
         <v>398</v>
       </c>
       <c r="F52">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G52">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H52" t="s">
         <v>399</v>
@@ -14440,10 +14440,10 @@
         <v>403</v>
       </c>
       <c r="F53">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G53">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="H53" t="s">
         <v>404</v>
@@ -14625,10 +14625,10 @@
         <v>380</v>
       </c>
       <c r="F54">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G54">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H54" t="s">
         <v>415</v>
@@ -14810,10 +14810,10 @@
         <v>398</v>
       </c>
       <c r="F55">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G55">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H55" t="s">
         <v>100</v>
@@ -14995,10 +14995,10 @@
         <v>398</v>
       </c>
       <c r="F56">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G56">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H56" t="s">
         <v>426</v>
@@ -15180,10 +15180,10 @@
         <v>398</v>
       </c>
       <c r="F57">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G57">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H57" t="s">
         <v>415</v>
@@ -15365,10 +15365,10 @@
         <v>398</v>
       </c>
       <c r="F58">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G58">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H58" t="s">
         <v>100</v>
@@ -15550,7 +15550,7 @@
         <v>398</v>
       </c>
       <c r="F59">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G59">
         <v>12</v>
@@ -15735,10 +15735,10 @@
         <v>440</v>
       </c>
       <c r="F60">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G60">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H60" t="s">
         <v>441</v>
@@ -15920,10 +15920,10 @@
         <v>440</v>
       </c>
       <c r="F61">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G61">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H61" t="s">
         <v>139</v>
@@ -16105,10 +16105,10 @@
         <v>449</v>
       </c>
       <c r="F62">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G62">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H62" t="s">
         <v>450</v>
@@ -16290,10 +16290,10 @@
         <v>455</v>
       </c>
       <c r="F63">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G63">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H63" t="s">
         <v>456</v>
@@ -16475,10 +16475,10 @@
         <v>462</v>
       </c>
       <c r="F64">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G64">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H64" t="s">
         <v>463</v>
@@ -16660,10 +16660,10 @@
         <v>455</v>
       </c>
       <c r="F65">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G65">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H65" t="s">
         <v>468</v>
@@ -16845,10 +16845,10 @@
         <v>462</v>
       </c>
       <c r="F66">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G66">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H66" t="s">
         <v>189</v>
@@ -17030,10 +17030,10 @@
         <v>455</v>
       </c>
       <c r="F67">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G67">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H67" t="s">
         <v>468</v>
@@ -17215,10 +17215,10 @@
         <v>455</v>
       </c>
       <c r="F68">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G68">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H68" t="s">
         <v>468</v>
@@ -17400,10 +17400,10 @@
         <v>455</v>
       </c>
       <c r="F69">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G69">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H69" t="s">
         <v>468</v>
@@ -17585,7 +17585,7 @@
         <v>493</v>
       </c>
       <c r="F70">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G70">
         <v>0</v>
@@ -17770,10 +17770,10 @@
         <v>497</v>
       </c>
       <c r="F71">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G71">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="H71" t="s">
         <v>404</v>
@@ -17955,10 +17955,10 @@
         <v>497</v>
       </c>
       <c r="F72">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G72">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="H72" t="s">
         <v>404</v>
@@ -18140,10 +18140,10 @@
         <v>497</v>
       </c>
       <c r="F73">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G73">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="H73" t="s">
         <v>404</v>
@@ -18325,7 +18325,7 @@
         <v>462</v>
       </c>
       <c r="F74">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G74">
         <v>1</v>
@@ -18510,7 +18510,7 @@
         <v>462</v>
       </c>
       <c r="F75">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G75">
         <v>1</v>
@@ -18695,10 +18695,10 @@
         <v>493</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G76">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H76" t="s">
         <v>518</v>
@@ -18880,7 +18880,7 @@
         <v>493</v>
       </c>
       <c r="F77">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G77">
         <v>5</v>
@@ -19065,10 +19065,10 @@
         <v>493</v>
       </c>
       <c r="F78">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G78">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H78" t="s">
         <v>170</v>
@@ -19250,7 +19250,7 @@
         <v>493</v>
       </c>
       <c r="F79">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G79">
         <v>5</v>
@@ -19435,10 +19435,10 @@
         <v>462</v>
       </c>
       <c r="F80">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G80">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H80" t="s">
         <v>535</v>
@@ -19620,10 +19620,10 @@
         <v>493</v>
       </c>
       <c r="F81">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G81">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H81" t="s">
         <v>544</v>
@@ -19805,10 +19805,10 @@
         <v>493</v>
       </c>
       <c r="F82">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G82">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H82" t="s">
         <v>549</v>
@@ -19990,10 +19990,10 @@
         <v>493</v>
       </c>
       <c r="F83">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G83">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H83" t="s">
         <v>554</v>
@@ -20175,10 +20175,10 @@
         <v>493</v>
       </c>
       <c r="F84">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G84">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H84" t="s">
         <v>369</v>
@@ -20360,10 +20360,10 @@
         <v>561</v>
       </c>
       <c r="F85">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G85">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H85" t="s">
         <v>404</v>
@@ -20545,10 +20545,10 @@
         <v>561</v>
       </c>
       <c r="F86">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G86">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H86" t="s">
         <v>404</v>
@@ -20730,10 +20730,10 @@
         <v>561</v>
       </c>
       <c r="F87">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G87">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H87" t="s">
         <v>404</v>
@@ -20915,10 +20915,10 @@
         <v>561</v>
       </c>
       <c r="F88">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G88">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H88" t="s">
         <v>404</v>
@@ -21100,10 +21100,10 @@
         <v>561</v>
       </c>
       <c r="F89">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G89">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H89" t="s">
         <v>404</v>
@@ -21285,10 +21285,10 @@
         <v>561</v>
       </c>
       <c r="F90">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G90">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H90" t="s">
         <v>404</v>
@@ -21470,10 +21470,10 @@
         <v>561</v>
       </c>
       <c r="F91">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G91">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H91" t="s">
         <v>404</v>
@@ -21655,10 +21655,10 @@
         <v>561</v>
       </c>
       <c r="F92">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G92">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H92" t="s">
         <v>404</v>
@@ -21840,10 +21840,10 @@
         <v>561</v>
       </c>
       <c r="F93">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G93">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H93" t="s">
         <v>404</v>
@@ -22025,10 +22025,10 @@
         <v>561</v>
       </c>
       <c r="F94">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G94">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H94" t="s">
         <v>404</v>
@@ -22210,10 +22210,10 @@
         <v>582</v>
       </c>
       <c r="F95">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G95">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H95" t="s">
         <v>583</v>
@@ -22395,10 +22395,10 @@
         <v>582</v>
       </c>
       <c r="F96">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G96">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H96" t="s">
         <v>588</v>
@@ -22580,10 +22580,10 @@
         <v>582</v>
       </c>
       <c r="F97">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G97">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H97" t="s">
         <v>369</v>
@@ -22765,10 +22765,10 @@
         <v>582</v>
       </c>
       <c r="F98">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G98">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H98" t="s">
         <v>599</v>
@@ -22950,10 +22950,10 @@
         <v>604</v>
       </c>
       <c r="F99">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G99">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H99" t="s">
         <v>605</v>
@@ -23135,10 +23135,10 @@
         <v>604</v>
       </c>
       <c r="F100">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G100">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H100" t="s">
         <v>605</v>
@@ -23320,10 +23320,10 @@
         <v>582</v>
       </c>
       <c r="F101">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G101">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H101" t="s">
         <v>613</v>
@@ -23505,10 +23505,10 @@
         <v>582</v>
       </c>
       <c r="F102">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G102">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H102" t="s">
         <v>617</v>
@@ -23690,10 +23690,10 @@
         <v>604</v>
       </c>
       <c r="F103">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G103">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H103" t="s">
         <v>622</v>
@@ -23875,10 +23875,10 @@
         <v>604</v>
       </c>
       <c r="F104">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G104">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H104" t="s">
         <v>626</v>
@@ -24060,10 +24060,10 @@
         <v>604</v>
       </c>
       <c r="F105">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G105">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H105" t="s">
         <v>622</v>
@@ -24245,10 +24245,10 @@
         <v>604</v>
       </c>
       <c r="F106">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G106">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H106" t="s">
         <v>631</v>
@@ -24430,10 +24430,10 @@
         <v>604</v>
       </c>
       <c r="F107">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G107">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H107" t="s">
         <v>100</v>
@@ -24615,10 +24615,10 @@
         <v>604</v>
       </c>
       <c r="F108">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G108">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H108" t="s">
         <v>636</v>
@@ -24800,10 +24800,10 @@
         <v>604</v>
       </c>
       <c r="F109">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G109">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H109" t="s">
         <v>640</v>
@@ -24985,10 +24985,10 @@
         <v>604</v>
       </c>
       <c r="F110">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G110">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H110" t="s">
         <v>605</v>
@@ -25170,10 +25170,10 @@
         <v>604</v>
       </c>
       <c r="F111">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G111">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H111" t="s">
         <v>648</v>
@@ -25355,10 +25355,10 @@
         <v>604</v>
       </c>
       <c r="F112">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G112">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H112" t="s">
         <v>655</v>
@@ -25540,10 +25540,10 @@
         <v>604</v>
       </c>
       <c r="F113">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G113">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H113" t="s">
         <v>345</v>
@@ -25725,10 +25725,10 @@
         <v>604</v>
       </c>
       <c r="F114">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G114">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H114" t="s">
         <v>345</v>
@@ -25910,10 +25910,10 @@
         <v>604</v>
       </c>
       <c r="F115">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G115">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H115" t="s">
         <v>665</v>
@@ -26095,10 +26095,10 @@
         <v>604</v>
       </c>
       <c r="F116">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G116">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H116" t="s">
         <v>671</v>
@@ -26280,10 +26280,10 @@
         <v>604</v>
       </c>
       <c r="F117">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G117">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H117" t="s">
         <v>677</v>
@@ -26465,10 +26465,10 @@
         <v>604</v>
       </c>
       <c r="F118">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G118">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H118" t="s">
         <v>685</v>
@@ -26650,10 +26650,10 @@
         <v>604</v>
       </c>
       <c r="F119">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G119">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H119" t="s">
         <v>691</v>
@@ -26835,10 +26835,10 @@
         <v>604</v>
       </c>
       <c r="F120">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G120">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H120" t="s">
         <v>554</v>
@@ -27020,10 +27020,10 @@
         <v>698</v>
       </c>
       <c r="F121">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G121">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H121" t="s">
         <v>699</v>
@@ -27205,10 +27205,10 @@
         <v>698</v>
       </c>
       <c r="F122">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G122">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H122" t="s">
         <v>665</v>
@@ -27390,10 +27390,10 @@
         <v>698</v>
       </c>
       <c r="F123">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G123">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H123" t="s">
         <v>87</v>
@@ -27575,7 +27575,7 @@
         <v>708</v>
       </c>
       <c r="F124">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G124">
         <v>4</v>
@@ -27760,7 +27760,7 @@
         <v>717</v>
       </c>
       <c r="F125">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G125">
         <v>1</v>
@@ -27945,10 +27945,10 @@
         <v>717</v>
       </c>
       <c r="F126">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G126">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H126" t="s">
         <v>724</v>
@@ -28130,10 +28130,10 @@
         <v>717</v>
       </c>
       <c r="F127">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G127">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H127" t="s">
         <v>728</v>
@@ -28315,10 +28315,10 @@
         <v>717</v>
       </c>
       <c r="F128">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G128">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H128" t="s">
         <v>456</v>
@@ -28500,10 +28500,10 @@
         <v>717</v>
       </c>
       <c r="F129">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G129">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H129" t="s">
         <v>736</v>
@@ -28685,10 +28685,10 @@
         <v>717</v>
       </c>
       <c r="F130">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G130">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H130" t="s">
         <v>744</v>
@@ -28870,10 +28870,10 @@
         <v>717</v>
       </c>
       <c r="F131">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G131">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H131" t="s">
         <v>750</v>
@@ -29055,10 +29055,10 @@
         <v>717</v>
       </c>
       <c r="F132">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G132">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H132" t="s">
         <v>755</v>
@@ -29240,10 +29240,10 @@
         <v>717</v>
       </c>
       <c r="F133">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G133">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H133" t="s">
         <v>287</v>
@@ -29425,10 +29425,10 @@
         <v>717</v>
       </c>
       <c r="F134">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G134">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H134" t="s">
         <v>762</v>
@@ -29610,10 +29610,10 @@
         <v>766</v>
       </c>
       <c r="F135">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G135">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H135" t="s">
         <v>767</v>
@@ -29795,10 +29795,10 @@
         <v>771</v>
       </c>
       <c r="F136">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G136">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H136" t="s">
         <v>404</v>
@@ -29980,10 +29980,10 @@
         <v>771</v>
       </c>
       <c r="F137">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G137">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H137" t="s">
         <v>404</v>
@@ -30165,10 +30165,10 @@
         <v>771</v>
       </c>
       <c r="F138">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G138">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H138" t="s">
         <v>404</v>
@@ -30350,10 +30350,10 @@
         <v>771</v>
       </c>
       <c r="F139">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G139">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H139" t="s">
         <v>404</v>
@@ -30535,10 +30535,10 @@
         <v>766</v>
       </c>
       <c r="F140">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G140">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H140" t="s">
         <v>280</v>
@@ -30720,10 +30720,10 @@
         <v>766</v>
       </c>
       <c r="F141">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G141">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H141" t="s">
         <v>280</v>
@@ -30905,10 +30905,10 @@
         <v>771</v>
       </c>
       <c r="F142">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G142">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H142" t="s">
         <v>404</v>
@@ -31090,10 +31090,10 @@
         <v>771</v>
       </c>
       <c r="F143">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G143">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H143" t="s">
         <v>404</v>
@@ -31275,10 +31275,10 @@
         <v>771</v>
       </c>
       <c r="F144">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G144">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H144" t="s">
         <v>404</v>
@@ -31460,10 +31460,10 @@
         <v>771</v>
       </c>
       <c r="F145">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G145">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="H145" t="s">
         <v>404</v>
@@ -31645,10 +31645,10 @@
         <v>766</v>
       </c>
       <c r="F146">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G146">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H146" t="s">
         <v>797</v>
@@ -31830,10 +31830,10 @@
         <v>766</v>
       </c>
       <c r="F147">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G147">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H147" t="s">
         <v>803</v>
@@ -32015,10 +32015,10 @@
         <v>766</v>
       </c>
       <c r="F148">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G148">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H148" t="s">
         <v>665</v>
@@ -32200,10 +32200,10 @@
         <v>717</v>
       </c>
       <c r="F149">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G149">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H149" t="s">
         <v>809</v>
@@ -32385,10 +32385,10 @@
         <v>717</v>
       </c>
       <c r="F150">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G150">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H150" t="s">
         <v>816</v>
@@ -32570,10 +32570,10 @@
         <v>766</v>
       </c>
       <c r="F151">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G151">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H151" t="s">
         <v>685</v>
@@ -32755,10 +32755,10 @@
         <v>766</v>
       </c>
       <c r="F152">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G152">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H152" t="s">
         <v>827</v>
@@ -32940,10 +32940,10 @@
         <v>766</v>
       </c>
       <c r="F153">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G153">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H153" t="s">
         <v>254</v>
@@ -33125,7 +33125,7 @@
         <v>717</v>
       </c>
       <c r="F154">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G154">
         <v>2</v>
@@ -33310,10 +33310,10 @@
         <v>766</v>
       </c>
       <c r="F155">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G155">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H155" t="s">
         <v>835</v>
@@ -33495,10 +33495,10 @@
         <v>766</v>
       </c>
       <c r="F156">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G156">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H156" t="s">
         <v>835</v>
@@ -33680,10 +33680,10 @@
         <v>766</v>
       </c>
       <c r="F157">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G157">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H157" t="s">
         <v>835</v>
@@ -33865,10 +33865,10 @@
         <v>766</v>
       </c>
       <c r="F158">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G158">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H158" t="s">
         <v>843</v>
@@ -34050,10 +34050,10 @@
         <v>766</v>
       </c>
       <c r="F159">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G159">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H159" t="s">
         <v>835</v>
@@ -34235,7 +34235,7 @@
         <v>766</v>
       </c>
       <c r="F160">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G160">
         <v>1</v>
@@ -34420,7 +34420,7 @@
         <v>766</v>
       </c>
       <c r="F161">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G161">
         <v>1</v>
@@ -34605,10 +34605,10 @@
         <v>766</v>
       </c>
       <c r="F162">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G162">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H162" t="s">
         <v>87</v>
@@ -34790,10 +34790,10 @@
         <v>766</v>
       </c>
       <c r="F163">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G163">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H163" t="s">
         <v>87</v>
@@ -34975,10 +34975,10 @@
         <v>860</v>
       </c>
       <c r="F164">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G164">
-        <v>-17</v>
+        <v>-15</v>
       </c>
       <c r="H164" t="s">
         <v>404</v>
@@ -35160,10 +35160,10 @@
         <v>863</v>
       </c>
       <c r="F165">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G165">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H165" t="s">
         <v>113</v>
@@ -35345,10 +35345,10 @@
         <v>766</v>
       </c>
       <c r="F166">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G166">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H166" t="s">
         <v>636</v>
@@ -35530,10 +35530,10 @@
         <v>766</v>
       </c>
       <c r="F167">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G167">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H167" t="s">
         <v>636</v>
@@ -35715,10 +35715,10 @@
         <v>863</v>
       </c>
       <c r="F168">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G168">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H168" t="s">
         <v>869</v>
@@ -35900,10 +35900,10 @@
         <v>766</v>
       </c>
       <c r="F169">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G169">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H169" t="s">
         <v>874</v>
@@ -36085,10 +36085,10 @@
         <v>766</v>
       </c>
       <c r="F170">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G170">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H170" t="s">
         <v>636</v>
@@ -36270,10 +36270,10 @@
         <v>863</v>
       </c>
       <c r="F171">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G171">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H171" t="s">
         <v>869</v>
@@ -36455,10 +36455,10 @@
         <v>863</v>
       </c>
       <c r="F172">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G172">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H172" t="s">
         <v>880</v>
@@ -36640,10 +36640,10 @@
         <v>863</v>
       </c>
       <c r="F173">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H173" t="s">
         <v>885</v>
@@ -36825,10 +36825,10 @@
         <v>863</v>
       </c>
       <c r="F174">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G174">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H174" t="s">
         <v>554</v>
@@ -37010,7 +37010,7 @@
         <v>863</v>
       </c>
       <c r="F175">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G175">
         <v>0</v>
@@ -37195,10 +37195,10 @@
         <v>766</v>
       </c>
       <c r="F176">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G176">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H176" t="s">
         <v>893</v>
@@ -37380,10 +37380,10 @@
         <v>863</v>
       </c>
       <c r="F177">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G177">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H177" t="s">
         <v>897</v>
@@ -37565,10 +37565,10 @@
         <v>766</v>
       </c>
       <c r="F178">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G178">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H178" t="s">
         <v>900</v>
@@ -37750,10 +37750,10 @@
         <v>863</v>
       </c>
       <c r="F179">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G179">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H179" t="s">
         <v>797</v>
@@ -37935,10 +37935,10 @@
         <v>863</v>
       </c>
       <c r="F180">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G180">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H180" t="s">
         <v>910</v>
@@ -38120,10 +38120,10 @@
         <v>863</v>
       </c>
       <c r="F181">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G181">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H181" t="s">
         <v>914</v>
@@ -38305,10 +38305,10 @@
         <v>863</v>
       </c>
       <c r="F182">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G182">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H182" t="s">
         <v>920</v>
@@ -38490,10 +38490,10 @@
         <v>863</v>
       </c>
       <c r="F183">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G183">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H183" t="s">
         <v>926</v>
@@ -38675,10 +38675,10 @@
         <v>863</v>
       </c>
       <c r="F184">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G184">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H184" t="s">
         <v>920</v>
@@ -38860,10 +38860,10 @@
         <v>863</v>
       </c>
       <c r="F185">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G185">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H185" t="s">
         <v>932</v>
@@ -39045,10 +39045,10 @@
         <v>863</v>
       </c>
       <c r="F186">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G186">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H186" t="s">
         <v>938</v>
@@ -39230,10 +39230,10 @@
         <v>863</v>
       </c>
       <c r="F187">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G187">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H187" t="s">
         <v>944</v>
@@ -39415,10 +39415,10 @@
         <v>863</v>
       </c>
       <c r="F188">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G188">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H188" t="s">
         <v>944</v>
@@ -39600,10 +39600,10 @@
         <v>863</v>
       </c>
       <c r="F189">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G189">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H189" t="s">
         <v>944</v>
@@ -39785,10 +39785,10 @@
         <v>863</v>
       </c>
       <c r="F190">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G190">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H190" t="s">
         <v>952</v>
@@ -39970,10 +39970,10 @@
         <v>956</v>
       </c>
       <c r="F191">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G191">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H191" t="s">
         <v>404</v>
@@ -40155,10 +40155,10 @@
         <v>956</v>
       </c>
       <c r="F192">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G192">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H192" t="s">
         <v>404</v>
@@ -40340,10 +40340,10 @@
         <v>956</v>
       </c>
       <c r="F193">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G193">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H193" t="s">
         <v>404</v>
@@ -40525,10 +40525,10 @@
         <v>956</v>
       </c>
       <c r="F194">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G194">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H194" t="s">
         <v>404</v>
@@ -40710,10 +40710,10 @@
         <v>956</v>
       </c>
       <c r="F195">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G195">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H195" t="s">
         <v>404</v>
@@ -40895,10 +40895,10 @@
         <v>956</v>
       </c>
       <c r="F196">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G196">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H196" t="s">
         <v>404</v>
@@ -41080,10 +41080,10 @@
         <v>956</v>
       </c>
       <c r="F197">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G197">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H197" t="s">
         <v>404</v>
@@ -41265,10 +41265,10 @@
         <v>956</v>
       </c>
       <c r="F198">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G198">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H198" t="s">
         <v>404</v>
@@ -41450,10 +41450,10 @@
         <v>863</v>
       </c>
       <c r="F199">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G199">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H199" t="s">
         <v>287</v>
@@ -41635,10 +41635,10 @@
         <v>956</v>
       </c>
       <c r="F200">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G200">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H200" t="s">
         <v>404</v>
@@ -41820,10 +41820,10 @@
         <v>956</v>
       </c>
       <c r="F201">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G201">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H201" t="s">
         <v>404</v>
@@ -42005,10 +42005,10 @@
         <v>863</v>
       </c>
       <c r="F202">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G202">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H202" t="s">
         <v>979</v>
@@ -42190,10 +42190,10 @@
         <v>863</v>
       </c>
       <c r="F203">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G203">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H203" t="s">
         <v>441</v>
@@ -42375,10 +42375,10 @@
         <v>863</v>
       </c>
       <c r="F204">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G204">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H204" t="s">
         <v>983</v>
@@ -42560,10 +42560,10 @@
         <v>863</v>
       </c>
       <c r="F205">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G205">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H205" t="s">
         <v>983</v>
@@ -42745,10 +42745,10 @@
         <v>863</v>
       </c>
       <c r="F206">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G206">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H206" t="s">
         <v>989</v>
@@ -42930,10 +42930,10 @@
         <v>863</v>
       </c>
       <c r="F207">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G207">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H207" t="s">
         <v>994</v>
@@ -43115,10 +43115,10 @@
         <v>863</v>
       </c>
       <c r="F208">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G208">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H208" t="s">
         <v>989</v>
@@ -43300,10 +43300,10 @@
         <v>1001</v>
       </c>
       <c r="F209">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G209">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H209" t="s">
         <v>583</v>
@@ -43485,10 +43485,10 @@
         <v>1001</v>
       </c>
       <c r="F210">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G210">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H210" t="s">
         <v>456</v>
@@ -43670,10 +43670,10 @@
         <v>863</v>
       </c>
       <c r="F211">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G211">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H211" t="s">
         <v>1005</v>
@@ -43855,10 +43855,10 @@
         <v>1001</v>
       </c>
       <c r="F212">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G212">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H212" t="s">
         <v>1012</v>
@@ -44040,10 +44040,10 @@
         <v>1001</v>
       </c>
       <c r="F213">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G213">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H213" t="s">
         <v>724</v>
@@ -44225,10 +44225,10 @@
         <v>1001</v>
       </c>
       <c r="F214">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G214">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H214" t="s">
         <v>724</v>
@@ -44410,10 +44410,10 @@
         <v>1001</v>
       </c>
       <c r="F215">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G215">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H215" t="s">
         <v>724</v>
@@ -44595,10 +44595,10 @@
         <v>1001</v>
       </c>
       <c r="F216">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G216">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H216" t="s">
         <v>724</v>
@@ -44780,10 +44780,10 @@
         <v>1001</v>
       </c>
       <c r="F217">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G217">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H217" t="s">
         <v>254</v>
@@ -44965,10 +44965,10 @@
         <v>1001</v>
       </c>
       <c r="F218">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G218">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H218" t="s">
         <v>920</v>
@@ -45150,10 +45150,10 @@
         <v>863</v>
       </c>
       <c r="F219">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G219">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H219" t="s">
         <v>391</v>
@@ -45335,10 +45335,10 @@
         <v>863</v>
       </c>
       <c r="F220">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G220">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H220" t="s">
         <v>1029</v>
@@ -45520,10 +45520,10 @@
         <v>863</v>
       </c>
       <c r="F221">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G221">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H221" t="s">
         <v>1029</v>
@@ -45705,10 +45705,10 @@
         <v>1001</v>
       </c>
       <c r="F222">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G222">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H222" t="s">
         <v>728</v>
@@ -45890,10 +45890,10 @@
         <v>1001</v>
       </c>
       <c r="F223">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G223">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H223" t="s">
         <v>728</v>
@@ -46075,10 +46075,10 @@
         <v>1001</v>
       </c>
       <c r="F224">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G224">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H224" t="s">
         <v>1047</v>
@@ -46260,10 +46260,10 @@
         <v>863</v>
       </c>
       <c r="F225">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G225">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H225" t="s">
         <v>1053</v>
@@ -46445,10 +46445,10 @@
         <v>1001</v>
       </c>
       <c r="F226">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G226">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H226" t="s">
         <v>724</v>
@@ -46630,10 +46630,10 @@
         <v>1001</v>
       </c>
       <c r="F227">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G227">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H227" t="s">
         <v>724</v>
@@ -46815,10 +46815,10 @@
         <v>863</v>
       </c>
       <c r="F228">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G228">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H228" t="s">
         <v>1047</v>
@@ -47000,10 +47000,10 @@
         <v>863</v>
       </c>
       <c r="F229">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G229">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H229" t="s">
         <v>1047</v>
@@ -47185,10 +47185,10 @@
         <v>1001</v>
       </c>
       <c r="F230">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G230">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H230" t="s">
         <v>1012</v>
@@ -47370,10 +47370,10 @@
         <v>1001</v>
       </c>
       <c r="F231">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G231">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H231" t="s">
         <v>1067</v>
@@ -47555,10 +47555,10 @@
         <v>863</v>
       </c>
       <c r="F232">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G232">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H232" t="s">
         <v>1072</v>
@@ -47740,10 +47740,10 @@
         <v>1001</v>
       </c>
       <c r="F233">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G233">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H233" t="s">
         <v>1076</v>
@@ -47925,10 +47925,10 @@
         <v>1001</v>
       </c>
       <c r="F234">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G234">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H234" t="s">
         <v>1081</v>
@@ -48110,10 +48110,10 @@
         <v>1001</v>
       </c>
       <c r="F235">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G235">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H235" t="s">
         <v>1085</v>
@@ -48295,10 +48295,10 @@
         <v>1001</v>
       </c>
       <c r="F236">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G236">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H236" t="s">
         <v>1081</v>
@@ -48480,10 +48480,10 @@
         <v>1001</v>
       </c>
       <c r="F237">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G237">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H237" t="s">
         <v>1092</v>
@@ -48665,10 +48665,10 @@
         <v>1001</v>
       </c>
       <c r="F238">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G238">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H238" t="s">
         <v>744</v>
@@ -48850,10 +48850,10 @@
         <v>1001</v>
       </c>
       <c r="F239">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G239">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H239" t="s">
         <v>1081</v>
@@ -49035,10 +49035,10 @@
         <v>863</v>
       </c>
       <c r="F240">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G240">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H240" t="s">
         <v>1100</v>
@@ -49220,10 +49220,10 @@
         <v>1001</v>
       </c>
       <c r="F241">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G241">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H241" t="s">
         <v>1105</v>
@@ -49405,10 +49405,10 @@
         <v>863</v>
       </c>
       <c r="F242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H242" t="s">
         <v>1029</v>
@@ -49590,10 +49590,10 @@
         <v>1001</v>
       </c>
       <c r="F243">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G243">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H243" t="s">
         <v>665</v>
@@ -49775,10 +49775,10 @@
         <v>1001</v>
       </c>
       <c r="F244">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G244">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H244" t="s">
         <v>66</v>
@@ -49960,10 +49960,10 @@
         <v>1001</v>
       </c>
       <c r="F245">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G245">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H245" t="s">
         <v>1121</v>
@@ -50145,10 +50145,10 @@
         <v>1001</v>
       </c>
       <c r="F246">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G246">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H246" t="s">
         <v>920</v>
@@ -50330,10 +50330,10 @@
         <v>1001</v>
       </c>
       <c r="F247">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G247">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H247" t="s">
         <v>1129</v>
@@ -50515,10 +50515,10 @@
         <v>1001</v>
       </c>
       <c r="F248">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G248">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H248" t="s">
         <v>1135</v>
@@ -50700,10 +50700,10 @@
         <v>1140</v>
       </c>
       <c r="F249">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G249">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H249" t="s">
         <v>583</v>
@@ -50885,10 +50885,10 @@
         <v>1140</v>
       </c>
       <c r="F250">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G250">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H250" t="s">
         <v>583</v>
@@ -51070,10 +51070,10 @@
         <v>1140</v>
       </c>
       <c r="F251">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G251">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H251" t="s">
         <v>1144</v>
@@ -51255,10 +51255,10 @@
         <v>1140</v>
       </c>
       <c r="F252">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G252">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H252" t="s">
         <v>531</v>
@@ -51440,10 +51440,10 @@
         <v>1153</v>
       </c>
       <c r="F253">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G253">
-        <v>-19</v>
+        <v>-17</v>
       </c>
       <c r="H253" t="s">
         <v>404</v>
@@ -51625,10 +51625,10 @@
         <v>1140</v>
       </c>
       <c r="F254">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G254">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H254" t="s">
         <v>1158</v>
@@ -51810,10 +51810,10 @@
         <v>1140</v>
       </c>
       <c r="F255">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G255">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H255" t="s">
         <v>1164</v>
@@ -51995,10 +51995,10 @@
         <v>1140</v>
       </c>
       <c r="F256">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G256">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H256" t="s">
         <v>1164</v>
@@ -52180,10 +52180,10 @@
         <v>1140</v>
       </c>
       <c r="F257">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G257">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H257" t="s">
         <v>518</v>
@@ -52365,10 +52365,10 @@
         <v>1140</v>
       </c>
       <c r="F258">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G258">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H258" t="s">
         <v>199</v>
@@ -52550,10 +52550,10 @@
         <v>1140</v>
       </c>
       <c r="F259">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G259">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H259" t="s">
         <v>1175</v>
@@ -52735,10 +52735,10 @@
         <v>1140</v>
       </c>
       <c r="F260">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G260">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H260" t="s">
         <v>1180</v>
@@ -52920,10 +52920,10 @@
         <v>1140</v>
       </c>
       <c r="F261">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G261">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H261" t="s">
         <v>1184</v>
@@ -53105,10 +53105,10 @@
         <v>1140</v>
       </c>
       <c r="F262">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G262">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H262" t="s">
         <v>989</v>
@@ -53290,10 +53290,10 @@
         <v>1140</v>
       </c>
       <c r="F263">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G263">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H263" t="s">
         <v>1192</v>
@@ -53475,10 +53475,10 @@
         <v>1140</v>
       </c>
       <c r="F264">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G264">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H264" t="s">
         <v>1197</v>
@@ -53660,10 +53660,10 @@
         <v>1140</v>
       </c>
       <c r="F265">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G265">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H265" t="s">
         <v>1202</v>
@@ -53845,10 +53845,10 @@
         <v>1140</v>
       </c>
       <c r="F266">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G266">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H266" t="s">
         <v>952</v>
@@ -54030,10 +54030,10 @@
         <v>1140</v>
       </c>
       <c r="F267">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G267">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H267" t="s">
         <v>1209</v>
@@ -54215,10 +54215,10 @@
         <v>1140</v>
       </c>
       <c r="F268">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G268">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H268" t="s">
         <v>1214</v>
@@ -54400,10 +54400,10 @@
         <v>1001</v>
       </c>
       <c r="F269">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G269">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H269" t="s">
         <v>1029</v>
@@ -54585,10 +54585,10 @@
         <v>1140</v>
       </c>
       <c r="F270">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G270">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H270" t="s">
         <v>1227</v>
@@ -54770,10 +54770,10 @@
         <v>1140</v>
       </c>
       <c r="F271">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G271">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H271" t="s">
         <v>1081</v>
@@ -54955,10 +54955,10 @@
         <v>1140</v>
       </c>
       <c r="F272">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G272">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H272" t="s">
         <v>1234</v>
@@ -55140,10 +55140,10 @@
         <v>1140</v>
       </c>
       <c r="F273">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G273">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H273" t="s">
         <v>750</v>
@@ -55325,10 +55325,10 @@
         <v>1140</v>
       </c>
       <c r="F274">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G274">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H274" t="s">
         <v>1238</v>
@@ -55510,10 +55510,10 @@
         <v>1001</v>
       </c>
       <c r="F275">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G275">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H275" t="s">
         <v>211</v>
@@ -55695,10 +55695,10 @@
         <v>1001</v>
       </c>
       <c r="F276">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G276">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H276" t="s">
         <v>211</v>
@@ -55880,10 +55880,10 @@
         <v>1140</v>
       </c>
       <c r="F277">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G277">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H277" t="s">
         <v>1238</v>
@@ -56065,10 +56065,10 @@
         <v>1001</v>
       </c>
       <c r="F278">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G278">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H278" t="s">
         <v>1100</v>
@@ -56250,10 +56250,10 @@
         <v>1140</v>
       </c>
       <c r="F279">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G279">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H279" t="s">
         <v>1247</v>
@@ -56435,10 +56435,10 @@
         <v>1140</v>
       </c>
       <c r="F280">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G280">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H280" t="s">
         <v>1250</v>
@@ -56620,10 +56620,10 @@
         <v>1140</v>
       </c>
       <c r="F281">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G281">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H281" t="s">
         <v>1250</v>
@@ -56805,10 +56805,10 @@
         <v>1140</v>
       </c>
       <c r="F282">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G282">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H282" t="s">
         <v>456</v>
@@ -56990,10 +56990,10 @@
         <v>1140</v>
       </c>
       <c r="F283">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G283">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H283" t="s">
         <v>1255</v>
@@ -57175,10 +57175,10 @@
         <v>1140</v>
       </c>
       <c r="F284">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G284">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H284" t="s">
         <v>1255</v>
@@ -57360,10 +57360,10 @@
         <v>1140</v>
       </c>
       <c r="F285">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G285">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H285" t="s">
         <v>456</v>
@@ -57545,10 +57545,10 @@
         <v>1261</v>
       </c>
       <c r="F286">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G286">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="H286" t="s">
         <v>404</v>
@@ -57730,10 +57730,10 @@
         <v>1140</v>
       </c>
       <c r="F287">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G287">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H287" t="s">
         <v>835</v>
@@ -57915,10 +57915,10 @@
         <v>1140</v>
       </c>
       <c r="F288">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G288">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H288" t="s">
         <v>835</v>
@@ -58100,10 +58100,10 @@
         <v>1140</v>
       </c>
       <c r="F289">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G289">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H289" t="s">
         <v>755</v>
@@ -58285,10 +58285,10 @@
         <v>1001</v>
       </c>
       <c r="F290">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G290">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H290" t="s">
         <v>1029</v>
@@ -58470,10 +58470,10 @@
         <v>1140</v>
       </c>
       <c r="F291">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G291">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H291" t="s">
         <v>1273</v>
@@ -58655,10 +58655,10 @@
         <v>1140</v>
       </c>
       <c r="F292">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G292">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H292" t="s">
         <v>797</v>
@@ -58840,10 +58840,10 @@
         <v>1140</v>
       </c>
       <c r="F293">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G293">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H293" t="s">
         <v>728</v>
@@ -59025,10 +59025,10 @@
         <v>1140</v>
       </c>
       <c r="F294">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G294">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H294" t="s">
         <v>1280</v>
@@ -59210,10 +59210,10 @@
         <v>1140</v>
       </c>
       <c r="F295">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G295">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H295" t="s">
         <v>170</v>
@@ -59395,10 +59395,10 @@
         <v>1140</v>
       </c>
       <c r="F296">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G296">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H296" t="s">
         <v>170</v>
@@ -59580,10 +59580,10 @@
         <v>1140</v>
       </c>
       <c r="F297">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G297">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H297" t="s">
         <v>691</v>
@@ -59765,10 +59765,10 @@
         <v>1001</v>
       </c>
       <c r="F298">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G298">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H298" t="s">
         <v>1287</v>
@@ -59950,10 +59950,10 @@
         <v>1140</v>
       </c>
       <c r="F299">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G299">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H299" t="s">
         <v>1293</v>
@@ -60135,10 +60135,10 @@
         <v>1140</v>
       </c>
       <c r="F300">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G300">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H300" t="s">
         <v>1293</v>
@@ -60320,10 +60320,10 @@
         <v>1140</v>
       </c>
       <c r="F301">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G301">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H301" t="s">
         <v>1300</v>
@@ -60505,10 +60505,10 @@
         <v>1001</v>
       </c>
       <c r="F302">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G302">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H302" t="s">
         <v>1306</v>
@@ -60690,10 +60690,10 @@
         <v>1001</v>
       </c>
       <c r="F303">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G303">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H303" t="s">
         <v>709</v>
@@ -60875,10 +60875,10 @@
         <v>1140</v>
       </c>
       <c r="F304">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G304">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H304" t="s">
         <v>1312</v>
@@ -61060,10 +61060,10 @@
         <v>1140</v>
       </c>
       <c r="F305">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G305">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H305" t="s">
         <v>1067</v>
@@ -61245,10 +61245,10 @@
         <v>1140</v>
       </c>
       <c r="F306">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G306">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H306" t="s">
         <v>1317</v>
@@ -61430,10 +61430,10 @@
         <v>1001</v>
       </c>
       <c r="F307">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G307">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H307" t="s">
         <v>1029</v>
@@ -61615,10 +61615,10 @@
         <v>1001</v>
       </c>
       <c r="F308">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G308">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H308" t="s">
         <v>415</v>
@@ -61800,10 +61800,10 @@
         <v>1001</v>
       </c>
       <c r="F309">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G309">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H309" t="s">
         <v>1327</v>
@@ -61985,10 +61985,10 @@
         <v>1001</v>
       </c>
       <c r="F310">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G310">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H310" t="s">
         <v>1029</v>
@@ -62170,10 +62170,10 @@
         <v>1001</v>
       </c>
       <c r="F311">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G311">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H311" t="s">
         <v>1341</v>
@@ -62355,10 +62355,10 @@
         <v>1001</v>
       </c>
       <c r="F312">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G312">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H312" t="s">
         <v>1100</v>
@@ -62540,10 +62540,10 @@
         <v>1140</v>
       </c>
       <c r="F313">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G313">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H313" t="s">
         <v>1348</v>
@@ -62725,10 +62725,10 @@
         <v>582</v>
       </c>
       <c r="F314">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G314">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H314" t="s">
         <v>337</v>
@@ -62910,10 +62910,10 @@
         <v>717</v>
       </c>
       <c r="F315">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G315">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H315" t="s">
         <v>1081</v>
@@ -63095,10 +63095,10 @@
         <v>717</v>
       </c>
       <c r="F316">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G316">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H316" t="s">
         <v>613</v>
@@ -63280,10 +63280,10 @@
         <v>863</v>
       </c>
       <c r="F317">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G317">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H317" t="s">
         <v>1360</v>
@@ -63465,10 +63465,10 @@
         <v>863</v>
       </c>
       <c r="F318">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G318">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H318" t="s">
         <v>1365</v>
@@ -63650,10 +63650,10 @@
         <v>863</v>
       </c>
       <c r="F319">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G319">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H319" t="s">
         <v>226</v>
@@ -63835,10 +63835,10 @@
         <v>863</v>
       </c>
       <c r="F320">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G320">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H320" t="s">
         <v>226</v>
@@ -64020,10 +64020,10 @@
         <v>863</v>
       </c>
       <c r="F321">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G321">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H321" t="s">
         <v>1375</v>
@@ -64205,7 +64205,7 @@
         <v>455</v>
       </c>
       <c r="F322">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G322">
         <v>9</v>
@@ -64390,7 +64390,7 @@
         <v>334</v>
       </c>
       <c r="F323">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G323">
         <v>12</v>
@@ -64575,10 +64575,10 @@
         <v>335</v>
       </c>
       <c r="F324">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G324">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H324" t="s">
         <v>199</v>
@@ -64760,10 +64760,10 @@
         <v>334</v>
       </c>
       <c r="F325">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G325">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H325" t="s">
         <v>1395</v>
@@ -64945,7 +64945,7 @@
         <v>380</v>
       </c>
       <c r="F326">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G326">
         <v>1</v>
@@ -65130,7 +65130,7 @@
         <v>455</v>
       </c>
       <c r="F327">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G327">
         <v>1</v>
@@ -65315,10 +65315,10 @@
         <v>493</v>
       </c>
       <c r="F328">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G328">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H328" t="s">
         <v>1404</v>
@@ -65500,10 +65500,10 @@
         <v>582</v>
       </c>
       <c r="F329">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G329">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H329" t="s">
         <v>599</v>
@@ -65685,10 +65685,10 @@
         <v>717</v>
       </c>
       <c r="F330">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G330">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H330" t="s">
         <v>426</v>
@@ -65870,10 +65870,10 @@
         <v>717</v>
       </c>
       <c r="F331">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G331">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H331" t="s">
         <v>1395</v>
@@ -66055,10 +66055,10 @@
         <v>766</v>
       </c>
       <c r="F332">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G332">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H332" t="s">
         <v>835</v>
@@ -66240,10 +66240,10 @@
         <v>766</v>
       </c>
       <c r="F333">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G333">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H333" t="s">
         <v>1414</v>
@@ -66425,10 +66425,10 @@
         <v>863</v>
       </c>
       <c r="F334">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G334">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H334" t="s">
         <v>1414</v>
@@ -66610,10 +66610,10 @@
         <v>1001</v>
       </c>
       <c r="F335">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G335">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H335" t="s">
         <v>1067</v>
@@ -66795,10 +66795,10 @@
         <v>1001</v>
       </c>
       <c r="F336">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G336">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H336" t="s">
         <v>1081</v>
@@ -66980,10 +66980,10 @@
         <v>1001</v>
       </c>
       <c r="F337">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G337">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H337" t="s">
         <v>1081</v>
@@ -67165,10 +67165,10 @@
         <v>1001</v>
       </c>
       <c r="F338">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G338">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H338" t="s">
         <v>1081</v>
@@ -67350,10 +67350,10 @@
         <v>1001</v>
       </c>
       <c r="F339">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G339">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H339" t="s">
         <v>1029</v>
@@ -67535,10 +67535,10 @@
         <v>1140</v>
       </c>
       <c r="F340">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G340">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H340" t="s">
         <v>1081</v>
@@ -67720,10 +67720,10 @@
         <v>1140</v>
       </c>
       <c r="F341">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G341">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H341" t="s">
         <v>835</v>
@@ -67905,10 +67905,10 @@
         <v>358</v>
       </c>
       <c r="F342">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G342">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H342" t="s">
         <v>1433</v>
@@ -68090,10 +68090,10 @@
         <v>717</v>
       </c>
       <c r="F343">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G343">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H343" t="s">
         <v>1005</v>
@@ -68275,10 +68275,10 @@
         <v>1001</v>
       </c>
       <c r="F344">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G344">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H344" t="s">
         <v>1433</v>
@@ -68460,10 +68460,10 @@
         <v>1001</v>
       </c>
       <c r="F345">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G345">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H345" t="s">
         <v>1433</v>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 26/10/2026 12:26:19
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{921C8F4E-9D68-4D6E-8FE6-C5AEDD80B88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E93364A0-B00B-426C-B034-644FFEC6F6AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{4E17D942-F2F4-4084-BE15-7C58A1BFC916}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{6DE24353-8926-402B-BA95-E792E85E264F}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4436,7 +4436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4A3FDDD-13CE-4741-B695-74CD079053C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849698AB-B5B4-4E59-8B69-025F8592FBB4}">
   <dimension ref="A1:BI298"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 27/10/2026 12:06:08
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1178C66D-02AE-4CFF-A9E1-8F5A8A3A89E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73B7113E-92DE-4284-A576-6392AEEC8CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{D7E0AB4D-B036-4008-92F3-8A78F74B312B}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{4DF55EDF-CF32-48AA-9D96-5834A7662657}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4935,7 +4935,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D41D5-A9A6-4D43-8036-9FC6362C53CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C3BC652-B017-4E08-875B-12006233F55B}">
   <dimension ref="A1:BI336"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 28/10/2026 12:55:38
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B465896E-DE86-4520-826E-EBCA25A8B4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2223EEA-3708-4191-9B38-0727898920F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{030031A3-29CE-4AA5-8E86-870DB26F359A}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0227B2E2-9820-4482-923F-21F0D07D7B74}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -5128,7 +5128,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB39ADCB-F30B-461D-AF90-6C4C1490B8D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D17EEE09-DE8A-476A-8EA1-42F19F3369EB}">
   <dimension ref="A1:BI362"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 28/10/2026 13:06:11
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2223EEA-3708-4191-9B38-0727898920F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BD0B9E9-60E4-4639-B337-C92391FAD35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0227B2E2-9820-4482-923F-21F0D07D7B74}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{B4C55F13-9E9D-40BE-A4A3-8EFE88523895}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -5128,7 +5128,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D17EEE09-DE8A-476A-8EA1-42F19F3369EB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8122FFA1-DC30-43A2-A293-E43B51B5E7FA}">
   <dimension ref="A1:BI362"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>